<commit_message>
Added a suitable PSU unit
</commit_message>
<xml_diff>
--- a/Components/PipettePuller/PipettePullerComponents.xlsx
+++ b/Components/PipettePuller/PipettePullerComponents.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gunet-my.sharepoint.com/personal/martin_selin_gu_se/Documents/PhD/Projects/DNA pulling/Pipette puller/Puller Githubg design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BF4A9E89-9ABB-47FD-A426-B06A4BA199B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8_{CAF44E09-7034-446B-B31E-A0E2CDA8DCF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22470" yWindow="0" windowWidth="16035" windowHeight="20985" xr2:uid="{04B1C45E-2BD0-4D38-9811-A8FC1AF4F80A}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="12120" xr2:uid="{04B1C45E-2BD0-4D38-9811-A8FC1AF4F80A}"/>
   </bookViews>
   <sheets>
     <sheet name="Pipette Puller components" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="39" uniqueCount="32">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="43" uniqueCount="36">
   <si>
     <t>3D print stl file</t>
   </si>
@@ -135,6 +135,18 @@
   </si>
   <si>
     <t>Name</t>
+  </si>
+  <si>
+    <t>Programmable Benchtop DC Power supply</t>
+  </si>
+  <si>
+    <t>TENMA 72-2540</t>
+  </si>
+  <si>
+    <t>Newark/Farnell</t>
+  </si>
+  <si>
+    <t>The provided software is compatible with TENMA power supplies, may need adapting for comaptability with other PSU units. PSU needs to be able to provide at least 4A.</t>
   </si>
 </sst>
 </file>
@@ -536,10 +548,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB6D0753-F963-4963-AC1B-C1A4D387C487}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.5703125" customWidth="1"/>
+    <col min="1" max="1" width="50.42578125" customWidth="1"/>
     <col min="2" max="2" width="23.140625" customWidth="1"/>
     <col min="3" max="3" width="20.28515625" customWidth="1"/>
     <col min="6" max="6" width="45.28515625" customWidth="1"/>
@@ -666,41 +678,41 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="1"/>
+    <row r="9" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>200</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10" t="s">
-        <v>1</v>
-      </c>
-      <c r="D10">
-        <v>2</v>
-      </c>
-      <c r="E10">
-        <v>1</v>
-      </c>
-      <c r="F10" t="s">
-        <v>0</v>
-      </c>
+      <c r="B10" s="1"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C11" t="s">
         <v>1</v>
       </c>
       <c r="D11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -711,10 +723,10 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B12" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C12" t="s">
         <v>1</v>
@@ -731,21 +743,41 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" t="s">
+        <v>1</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>3</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B14" t="s">
         <v>2</v>
       </c>
-      <c r="C13" t="s">
-        <v>1</v>
-      </c>
-      <c r="D13">
-        <v>1</v>
-      </c>
-      <c r="E13">
-        <v>1</v>
-      </c>
-      <c r="F13" t="s">
+      <c r="C14" t="s">
+        <v>1</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>